<commit_message>
[UPDATE]Remove Total Amount Column in Excel Sheet
</commit_message>
<xml_diff>
--- a/home_kouzina_sales/static/src/files/Sale_Orders.xlsx
+++ b/home_kouzina_sales/static/src/files/Sale_Orders.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="49">
   <si>
     <t xml:space="preserve">Marketplace Order ID</t>
   </si>
@@ -94,9 +94,6 @@
     <t xml:space="preserve">Delivery Slot</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Amount</t>
-  </si>
-  <si>
     <t xml:space="preserve">Invoice Number</t>
   </si>
   <si>
@@ -115,7 +112,7 @@
     <t xml:space="preserve">Item ID</t>
   </si>
   <si>
-    <t xml:space="preserve">MKP-1965445556711121015</t>
+    <t xml:space="preserve">MKP-19456667</t>
   </si>
   <si>
     <t xml:space="preserve">2026-05-28</t>
@@ -601,7 +598,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF5"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
@@ -625,11 +622,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="28" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="30" style="1" width="31.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="29" style="1" width="31.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -723,53 +720,50 @@
       <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AF1" s="5"/>
+      <c r="AE1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="I2" s="7" t="n">
         <v>400001</v>
       </c>
       <c r="J2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="M2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>42</v>
       </c>
       <c r="O2" s="7" t="n">
         <v>1</v>
@@ -785,43 +779,40 @@
         <v>0</v>
       </c>
       <c r="T2" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="V2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="U2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="V2" s="6" t="s">
+      <c r="W2" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="W2" s="6" t="s">
+      <c r="X2" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="X2" s="6" t="s">
+      <c r="Y2" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="Y2" s="7" t="n">
-        <v>100</v>
       </c>
       <c r="Z2" s="6" t="s">
         <v>47</v>
       </c>
       <c r="AA2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="AB2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AC2" s="6" t="s">
-        <v>49</v>
+      <c r="AC2" s="6" t="n">
+        <v>123456</v>
       </c>
       <c r="AD2" s="6" t="n">
-        <v>123456</v>
-      </c>
-      <c r="AE2" s="6" t="n">
         <v>43</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="6"/>
       <c r="D3" s="6"/>
       <c r="G3" s="6"/>
@@ -837,13 +828,12 @@
       <c r="V3" s="6"/>
       <c r="W3" s="5"/>
       <c r="X3" s="6"/>
-      <c r="Y3" s="7"/>
+      <c r="Y3" s="6"/>
       <c r="Z3" s="6"/>
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="R4" s="7"/>

</xml_diff>